<commit_message>
Jobber videre med befolkning per opptaksområde
</commit_message>
<xml_diff>
--- a/Opptaksområder/KLASS PHV/OPPTAK_PHV_2018.xlsx
+++ b/Opptaksområder/KLASS PHV/OPPTAK_PHV_2018.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="477">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="478">
   <si>
     <t xml:space="preserve">KOMMUNE</t>
   </si>
@@ -197,15 +197,15 @@
     <t xml:space="preserve">0402</t>
   </si>
   <si>
+    <t xml:space="preserve">983971709</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SYKEHUSET INNLANDET HF</t>
+  </si>
+  <si>
     <t xml:space="preserve">0403</t>
   </si>
   <si>
-    <t xml:space="preserve">983971709</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SYKEHUSET INNLANDET HF</t>
-  </si>
-  <si>
     <t xml:space="preserve">0412</t>
   </si>
   <si>
@@ -875,6 +875,15 @@
     <t xml:space="preserve">1444</t>
   </si>
   <si>
+    <t xml:space="preserve">1445</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1449</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1502</t>
+  </si>
+  <si>
     <t xml:space="preserve">997005562</t>
   </si>
   <si>
@@ -887,15 +896,6 @@
     <t xml:space="preserve">HELSE MIDT-NORGE RHF</t>
   </si>
   <si>
-    <t xml:space="preserve">1445</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1449</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1502</t>
-  </si>
-  <si>
     <t xml:space="preserve">1504</t>
   </si>
   <si>
@@ -1337,112 +1337,115 @@
     <t xml:space="preserve">5018</t>
   </si>
   <si>
+    <t xml:space="preserve">5020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5049</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5054</t>
+  </si>
+  <si>
     <t xml:space="preserve">5019</t>
   </si>
   <si>
-    <t xml:space="preserve">5020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5029</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5030</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5033</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5034</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5036</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5037</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5038</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5039</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5040</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5042</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5043</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5044</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5045</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5046</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5047</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5048</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5049</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5050</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5051</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5052</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5053</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5054</t>
+    <t xml:space="preserve">5061</t>
   </si>
 </sst>
 </file>
@@ -2099,10 +2102,10 @@
         <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="C20" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="D20" t="s">
         <v>8</v>
@@ -2541,10 +2544,10 @@
         <v>60</v>
       </c>
       <c r="B46" t="s">
-        <v>17</v>
+        <v>61</v>
       </c>
       <c r="C46" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="D46" t="s">
         <v>8</v>
@@ -2555,13 +2558,13 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
+        <v>63</v>
+      </c>
+      <c r="B47" t="s">
         <v>61</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>62</v>
-      </c>
-      <c r="C47" t="s">
-        <v>63</v>
       </c>
       <c r="D47" t="s">
         <v>8</v>
@@ -2575,10 +2578,10 @@
         <v>64</v>
       </c>
       <c r="B48" t="s">
+        <v>61</v>
+      </c>
+      <c r="C48" t="s">
         <v>62</v>
-      </c>
-      <c r="C48" t="s">
-        <v>63</v>
       </c>
       <c r="D48" t="s">
         <v>8</v>
@@ -2592,10 +2595,10 @@
         <v>65</v>
       </c>
       <c r="B49" t="s">
+        <v>61</v>
+      </c>
+      <c r="C49" t="s">
         <v>62</v>
-      </c>
-      <c r="C49" t="s">
-        <v>63</v>
       </c>
       <c r="D49" t="s">
         <v>8</v>
@@ -2609,10 +2612,10 @@
         <v>66</v>
       </c>
       <c r="B50" t="s">
+        <v>61</v>
+      </c>
+      <c r="C50" t="s">
         <v>62</v>
-      </c>
-      <c r="C50" t="s">
-        <v>63</v>
       </c>
       <c r="D50" t="s">
         <v>8</v>
@@ -2626,10 +2629,10 @@
         <v>67</v>
       </c>
       <c r="B51" t="s">
-        <v>17</v>
+        <v>61</v>
       </c>
       <c r="C51" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="D51" t="s">
         <v>8</v>
@@ -2643,10 +2646,10 @@
         <v>68</v>
       </c>
       <c r="B52" t="s">
-        <v>17</v>
+        <v>61</v>
       </c>
       <c r="C52" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="D52" t="s">
         <v>8</v>
@@ -2660,10 +2663,10 @@
         <v>69</v>
       </c>
       <c r="B53" t="s">
-        <v>17</v>
+        <v>61</v>
       </c>
       <c r="C53" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="D53" t="s">
         <v>8</v>
@@ -2677,10 +2680,10 @@
         <v>70</v>
       </c>
       <c r="B54" t="s">
-        <v>17</v>
+        <v>61</v>
       </c>
       <c r="C54" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="D54" t="s">
         <v>8</v>
@@ -2694,10 +2697,10 @@
         <v>71</v>
       </c>
       <c r="B55" t="s">
+        <v>61</v>
+      </c>
+      <c r="C55" t="s">
         <v>62</v>
-      </c>
-      <c r="C55" t="s">
-        <v>63</v>
       </c>
       <c r="D55" t="s">
         <v>8</v>
@@ -2711,10 +2714,10 @@
         <v>72</v>
       </c>
       <c r="B56" t="s">
+        <v>61</v>
+      </c>
+      <c r="C56" t="s">
         <v>62</v>
-      </c>
-      <c r="C56" t="s">
-        <v>63</v>
       </c>
       <c r="D56" t="s">
         <v>8</v>
@@ -2728,10 +2731,10 @@
         <v>73</v>
       </c>
       <c r="B57" t="s">
+        <v>61</v>
+      </c>
+      <c r="C57" t="s">
         <v>62</v>
-      </c>
-      <c r="C57" t="s">
-        <v>63</v>
       </c>
       <c r="D57" t="s">
         <v>8</v>
@@ -2745,10 +2748,10 @@
         <v>74</v>
       </c>
       <c r="B58" t="s">
+        <v>61</v>
+      </c>
+      <c r="C58" t="s">
         <v>62</v>
-      </c>
-      <c r="C58" t="s">
-        <v>63</v>
       </c>
       <c r="D58" t="s">
         <v>8</v>
@@ -2762,10 +2765,10 @@
         <v>75</v>
       </c>
       <c r="B59" t="s">
+        <v>61</v>
+      </c>
+      <c r="C59" t="s">
         <v>62</v>
-      </c>
-      <c r="C59" t="s">
-        <v>63</v>
       </c>
       <c r="D59" t="s">
         <v>8</v>
@@ -2779,10 +2782,10 @@
         <v>76</v>
       </c>
       <c r="B60" t="s">
+        <v>61</v>
+      </c>
+      <c r="C60" t="s">
         <v>62</v>
-      </c>
-      <c r="C60" t="s">
-        <v>63</v>
       </c>
       <c r="D60" t="s">
         <v>8</v>
@@ -2796,10 +2799,10 @@
         <v>77</v>
       </c>
       <c r="B61" t="s">
+        <v>61</v>
+      </c>
+      <c r="C61" t="s">
         <v>62</v>
-      </c>
-      <c r="C61" t="s">
-        <v>63</v>
       </c>
       <c r="D61" t="s">
         <v>8</v>
@@ -2813,10 +2816,10 @@
         <v>78</v>
       </c>
       <c r="B62" t="s">
+        <v>61</v>
+      </c>
+      <c r="C62" t="s">
         <v>62</v>
-      </c>
-      <c r="C62" t="s">
-        <v>63</v>
       </c>
       <c r="D62" t="s">
         <v>8</v>
@@ -2830,10 +2833,10 @@
         <v>79</v>
       </c>
       <c r="B63" t="s">
+        <v>61</v>
+      </c>
+      <c r="C63" t="s">
         <v>62</v>
-      </c>
-      <c r="C63" t="s">
-        <v>63</v>
       </c>
       <c r="D63" t="s">
         <v>8</v>
@@ -2847,10 +2850,10 @@
         <v>80</v>
       </c>
       <c r="B64" t="s">
+        <v>61</v>
+      </c>
+      <c r="C64" t="s">
         <v>62</v>
-      </c>
-      <c r="C64" t="s">
-        <v>63</v>
       </c>
       <c r="D64" t="s">
         <v>8</v>
@@ -2864,10 +2867,10 @@
         <v>81</v>
       </c>
       <c r="B65" t="s">
+        <v>61</v>
+      </c>
+      <c r="C65" t="s">
         <v>62</v>
-      </c>
-      <c r="C65" t="s">
-        <v>63</v>
       </c>
       <c r="D65" t="s">
         <v>8</v>
@@ -2881,10 +2884,10 @@
         <v>82</v>
       </c>
       <c r="B66" t="s">
+        <v>61</v>
+      </c>
+      <c r="C66" t="s">
         <v>62</v>
-      </c>
-      <c r="C66" t="s">
-        <v>63</v>
       </c>
       <c r="D66" t="s">
         <v>8</v>
@@ -2898,10 +2901,10 @@
         <v>83</v>
       </c>
       <c r="B67" t="s">
+        <v>61</v>
+      </c>
+      <c r="C67" t="s">
         <v>62</v>
-      </c>
-      <c r="C67" t="s">
-        <v>63</v>
       </c>
       <c r="D67" t="s">
         <v>8</v>
@@ -2915,10 +2918,10 @@
         <v>84</v>
       </c>
       <c r="B68" t="s">
+        <v>61</v>
+      </c>
+      <c r="C68" t="s">
         <v>62</v>
-      </c>
-      <c r="C68" t="s">
-        <v>63</v>
       </c>
       <c r="D68" t="s">
         <v>8</v>
@@ -2932,10 +2935,10 @@
         <v>85</v>
       </c>
       <c r="B69" t="s">
+        <v>61</v>
+      </c>
+      <c r="C69" t="s">
         <v>62</v>
-      </c>
-      <c r="C69" t="s">
-        <v>63</v>
       </c>
       <c r="D69" t="s">
         <v>8</v>
@@ -2949,10 +2952,10 @@
         <v>86</v>
       </c>
       <c r="B70" t="s">
+        <v>61</v>
+      </c>
+      <c r="C70" t="s">
         <v>62</v>
-      </c>
-      <c r="C70" t="s">
-        <v>63</v>
       </c>
       <c r="D70" t="s">
         <v>8</v>
@@ -2966,10 +2969,10 @@
         <v>87</v>
       </c>
       <c r="B71" t="s">
+        <v>61</v>
+      </c>
+      <c r="C71" t="s">
         <v>62</v>
-      </c>
-      <c r="C71" t="s">
-        <v>63</v>
       </c>
       <c r="D71" t="s">
         <v>8</v>
@@ -2983,10 +2986,10 @@
         <v>88</v>
       </c>
       <c r="B72" t="s">
+        <v>61</v>
+      </c>
+      <c r="C72" t="s">
         <v>62</v>
-      </c>
-      <c r="C72" t="s">
-        <v>63</v>
       </c>
       <c r="D72" t="s">
         <v>8</v>
@@ -3000,10 +3003,10 @@
         <v>89</v>
       </c>
       <c r="B73" t="s">
+        <v>61</v>
+      </c>
+      <c r="C73" t="s">
         <v>62</v>
-      </c>
-      <c r="C73" t="s">
-        <v>63</v>
       </c>
       <c r="D73" t="s">
         <v>8</v>
@@ -3017,10 +3020,10 @@
         <v>90</v>
       </c>
       <c r="B74" t="s">
+        <v>61</v>
+      </c>
+      <c r="C74" t="s">
         <v>62</v>
-      </c>
-      <c r="C74" t="s">
-        <v>63</v>
       </c>
       <c r="D74" t="s">
         <v>8</v>
@@ -3034,10 +3037,10 @@
         <v>91</v>
       </c>
       <c r="B75" t="s">
+        <v>61</v>
+      </c>
+      <c r="C75" t="s">
         <v>62</v>
-      </c>
-      <c r="C75" t="s">
-        <v>63</v>
       </c>
       <c r="D75" t="s">
         <v>8</v>
@@ -3051,10 +3054,10 @@
         <v>92</v>
       </c>
       <c r="B76" t="s">
+        <v>61</v>
+      </c>
+      <c r="C76" t="s">
         <v>62</v>
-      </c>
-      <c r="C76" t="s">
-        <v>63</v>
       </c>
       <c r="D76" t="s">
         <v>8</v>
@@ -3068,10 +3071,10 @@
         <v>93</v>
       </c>
       <c r="B77" t="s">
+        <v>61</v>
+      </c>
+      <c r="C77" t="s">
         <v>62</v>
-      </c>
-      <c r="C77" t="s">
-        <v>63</v>
       </c>
       <c r="D77" t="s">
         <v>8</v>
@@ -3085,10 +3088,10 @@
         <v>94</v>
       </c>
       <c r="B78" t="s">
+        <v>61</v>
+      </c>
+      <c r="C78" t="s">
         <v>62</v>
-      </c>
-      <c r="C78" t="s">
-        <v>63</v>
       </c>
       <c r="D78" t="s">
         <v>8</v>
@@ -3102,10 +3105,10 @@
         <v>95</v>
       </c>
       <c r="B79" t="s">
+        <v>61</v>
+      </c>
+      <c r="C79" t="s">
         <v>62</v>
-      </c>
-      <c r="C79" t="s">
-        <v>63</v>
       </c>
       <c r="D79" t="s">
         <v>8</v>
@@ -3119,10 +3122,10 @@
         <v>96</v>
       </c>
       <c r="B80" t="s">
+        <v>61</v>
+      </c>
+      <c r="C80" t="s">
         <v>62</v>
-      </c>
-      <c r="C80" t="s">
-        <v>63</v>
       </c>
       <c r="D80" t="s">
         <v>8</v>
@@ -3136,10 +3139,10 @@
         <v>97</v>
       </c>
       <c r="B81" t="s">
+        <v>61</v>
+      </c>
+      <c r="C81" t="s">
         <v>62</v>
-      </c>
-      <c r="C81" t="s">
-        <v>63</v>
       </c>
       <c r="D81" t="s">
         <v>8</v>
@@ -3153,10 +3156,10 @@
         <v>98</v>
       </c>
       <c r="B82" t="s">
+        <v>61</v>
+      </c>
+      <c r="C82" t="s">
         <v>62</v>
-      </c>
-      <c r="C82" t="s">
-        <v>63</v>
       </c>
       <c r="D82" t="s">
         <v>8</v>
@@ -3187,10 +3190,10 @@
         <v>100</v>
       </c>
       <c r="B84" t="s">
+        <v>61</v>
+      </c>
+      <c r="C84" t="s">
         <v>62</v>
-      </c>
-      <c r="C84" t="s">
-        <v>63</v>
       </c>
       <c r="D84" t="s">
         <v>8</v>
@@ -3204,10 +3207,10 @@
         <v>101</v>
       </c>
       <c r="B85" t="s">
+        <v>61</v>
+      </c>
+      <c r="C85" t="s">
         <v>62</v>
-      </c>
-      <c r="C85" t="s">
-        <v>63</v>
       </c>
       <c r="D85" t="s">
         <v>8</v>
@@ -3221,10 +3224,10 @@
         <v>102</v>
       </c>
       <c r="B86" t="s">
+        <v>61</v>
+      </c>
+      <c r="C86" t="s">
         <v>62</v>
-      </c>
-      <c r="C86" t="s">
-        <v>63</v>
       </c>
       <c r="D86" t="s">
         <v>8</v>
@@ -3238,10 +3241,10 @@
         <v>103</v>
       </c>
       <c r="B87" t="s">
+        <v>61</v>
+      </c>
+      <c r="C87" t="s">
         <v>62</v>
-      </c>
-      <c r="C87" t="s">
-        <v>63</v>
       </c>
       <c r="D87" t="s">
         <v>8</v>
@@ -3255,10 +3258,10 @@
         <v>104</v>
       </c>
       <c r="B88" t="s">
+        <v>61</v>
+      </c>
+      <c r="C88" t="s">
         <v>62</v>
-      </c>
-      <c r="C88" t="s">
-        <v>63</v>
       </c>
       <c r="D88" t="s">
         <v>8</v>
@@ -3272,10 +3275,10 @@
         <v>105</v>
       </c>
       <c r="B89" t="s">
+        <v>61</v>
+      </c>
+      <c r="C89" t="s">
         <v>62</v>
-      </c>
-      <c r="C89" t="s">
-        <v>63</v>
       </c>
       <c r="D89" t="s">
         <v>8</v>
@@ -3289,10 +3292,10 @@
         <v>106</v>
       </c>
       <c r="B90" t="s">
+        <v>61</v>
+      </c>
+      <c r="C90" t="s">
         <v>62</v>
-      </c>
-      <c r="C90" t="s">
-        <v>63</v>
       </c>
       <c r="D90" t="s">
         <v>8</v>
@@ -3306,10 +3309,10 @@
         <v>107</v>
       </c>
       <c r="B91" t="s">
+        <v>61</v>
+      </c>
+      <c r="C91" t="s">
         <v>62</v>
-      </c>
-      <c r="C91" t="s">
-        <v>63</v>
       </c>
       <c r="D91" t="s">
         <v>8</v>
@@ -3323,10 +3326,10 @@
         <v>108</v>
       </c>
       <c r="B92" t="s">
+        <v>61</v>
+      </c>
+      <c r="C92" t="s">
         <v>62</v>
-      </c>
-      <c r="C92" t="s">
-        <v>63</v>
       </c>
       <c r="D92" t="s">
         <v>8</v>
@@ -3340,10 +3343,10 @@
         <v>109</v>
       </c>
       <c r="B93" t="s">
+        <v>61</v>
+      </c>
+      <c r="C93" t="s">
         <v>62</v>
-      </c>
-      <c r="C93" t="s">
-        <v>63</v>
       </c>
       <c r="D93" t="s">
         <v>8</v>
@@ -5309,13 +5312,13 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B209" t="s">
-        <v>227</v>
+        <v>202</v>
       </c>
       <c r="C209" t="s">
-        <v>228</v>
+        <v>203</v>
       </c>
       <c r="D209" t="s">
         <v>197</v>
@@ -5326,13 +5329,13 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B210" t="s">
-        <v>202</v>
+        <v>227</v>
       </c>
       <c r="C210" t="s">
-        <v>203</v>
+        <v>228</v>
       </c>
       <c r="D210" t="s">
         <v>197</v>
@@ -5343,7 +5346,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B211" t="s">
         <v>227</v>
@@ -5360,7 +5363,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B212" t="s">
         <v>227</v>
@@ -5377,7 +5380,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B213" t="s">
         <v>227</v>
@@ -5394,7 +5397,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B214" t="s">
         <v>227</v>
@@ -5411,7 +5414,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B215" t="s">
         <v>227</v>
@@ -5428,7 +5431,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B216" t="s">
         <v>227</v>
@@ -5445,7 +5448,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B217" t="s">
         <v>227</v>
@@ -5462,7 +5465,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B218" t="s">
         <v>227</v>
@@ -5479,7 +5482,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B219" t="s">
         <v>227</v>
@@ -5496,7 +5499,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B220" t="s">
         <v>227</v>
@@ -5513,7 +5516,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B221" t="s">
         <v>227</v>
@@ -5530,7 +5533,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B222" t="s">
         <v>227</v>
@@ -5547,7 +5550,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B223" t="s">
         <v>227</v>
@@ -5564,7 +5567,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B224" t="s">
         <v>227</v>
@@ -5581,7 +5584,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B225" t="s">
         <v>227</v>
@@ -5598,7 +5601,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B226" t="s">
         <v>227</v>
@@ -5615,7 +5618,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B227" t="s">
         <v>227</v>
@@ -5632,7 +5635,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B228" t="s">
         <v>227</v>
@@ -5649,7 +5652,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B229" t="s">
         <v>227</v>
@@ -5666,7 +5669,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B230" t="s">
         <v>227</v>
@@ -5683,13 +5686,13 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B231" t="s">
-        <v>227</v>
+        <v>262</v>
       </c>
       <c r="C231" t="s">
-        <v>228</v>
+        <v>263</v>
       </c>
       <c r="D231" t="s">
         <v>197</v>
@@ -5700,13 +5703,13 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B232" t="s">
-        <v>262</v>
+        <v>227</v>
       </c>
       <c r="C232" t="s">
-        <v>263</v>
+        <v>228</v>
       </c>
       <c r="D232" t="s">
         <v>197</v>
@@ -5717,13 +5720,13 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B233" t="s">
-        <v>227</v>
+        <v>262</v>
       </c>
       <c r="C233" t="s">
-        <v>228</v>
+        <v>263</v>
       </c>
       <c r="D233" t="s">
         <v>197</v>
@@ -5734,7 +5737,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B234" t="s">
         <v>262</v>
@@ -5751,7 +5754,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B235" t="s">
         <v>262</v>
@@ -5768,7 +5771,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B236" t="s">
         <v>262</v>
@@ -5785,7 +5788,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B237" t="s">
         <v>262</v>
@@ -5802,7 +5805,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B238" t="s">
         <v>262</v>
@@ -5819,7 +5822,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B239" t="s">
         <v>262</v>
@@ -5836,7 +5839,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B240" t="s">
         <v>262</v>
@@ -5853,7 +5856,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B241" t="s">
         <v>262</v>
@@ -5870,7 +5873,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B242" t="s">
         <v>262</v>
@@ -5887,7 +5890,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B243" t="s">
         <v>262</v>
@@ -5904,7 +5907,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B244" t="s">
         <v>262</v>
@@ -5921,7 +5924,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B245" t="s">
         <v>262</v>
@@ -5938,7 +5941,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B246" t="s">
         <v>262</v>
@@ -5955,7 +5958,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B247" t="s">
         <v>262</v>
@@ -5972,7 +5975,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B248" t="s">
         <v>262</v>
@@ -5989,7 +5992,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B249" t="s">
         <v>262</v>
@@ -6006,7 +6009,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B250" t="s">
         <v>262</v>
@@ -6023,7 +6026,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B251" t="s">
         <v>262</v>
@@ -6040,7 +6043,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B252" t="s">
         <v>262</v>
@@ -6057,7 +6060,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B253" t="s">
         <v>262</v>
@@ -6074,7 +6077,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B254" t="s">
         <v>262</v>
@@ -6091,24 +6094,24 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B255" t="s">
-        <v>287</v>
+        <v>262</v>
       </c>
       <c r="C255" t="s">
-        <v>288</v>
+        <v>263</v>
       </c>
       <c r="D255" t="s">
-        <v>289</v>
+        <v>197</v>
       </c>
       <c r="E255" t="s">
-        <v>290</v>
+        <v>198</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="B256" t="s">
         <v>262</v>
@@ -6125,642 +6128,642 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
+        <v>289</v>
+      </c>
+      <c r="B257" t="s">
+        <v>290</v>
+      </c>
+      <c r="C257" t="s">
+        <v>291</v>
+      </c>
+      <c r="D257" t="s">
         <v>292</v>
       </c>
-      <c r="B257" t="s">
-        <v>262</v>
-      </c>
-      <c r="C257" t="s">
-        <v>263</v>
-      </c>
-      <c r="D257" t="s">
-        <v>197</v>
-      </c>
       <c r="E257" t="s">
-        <v>198</v>
+        <v>293</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="s">
+        <v>294</v>
+      </c>
+      <c r="B258" t="s">
+        <v>290</v>
+      </c>
+      <c r="C258" t="s">
+        <v>291</v>
+      </c>
+      <c r="D258" t="s">
+        <v>292</v>
+      </c>
+      <c r="E258" t="s">
         <v>293</v>
-      </c>
-      <c r="B258" t="s">
-        <v>287</v>
-      </c>
-      <c r="C258" t="s">
-        <v>288</v>
-      </c>
-      <c r="D258" t="s">
-        <v>289</v>
-      </c>
-      <c r="E258" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B259" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C259" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D259" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E259" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B260" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C260" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D260" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E260" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B261" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C261" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D261" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E261" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B262" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C262" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D262" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E262" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B263" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C263" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D263" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E263" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B264" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C264" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D264" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E264" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B265" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C265" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D265" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E265" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B266" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C266" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D266" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E266" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B267" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C267" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D267" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E267" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B268" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C268" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D268" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E268" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B269" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C269" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D269" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E269" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B270" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C270" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D270" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E270" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B271" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C271" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D271" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E271" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B272" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C272" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D272" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E272" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B273" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C273" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D273" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E273" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B274" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C274" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D274" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E274" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B275" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C275" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D275" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E275" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B276" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C276" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D276" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E276" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B277" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C277" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D277" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E277" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B278" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C278" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D278" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E278" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B279" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C279" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D279" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E279" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B280" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C280" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D280" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E280" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B281" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C281" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D281" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E281" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B282" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C282" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D282" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E282" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B283" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C283" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D283" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E283" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B284" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C284" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D284" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E284" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B285" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C285" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D285" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E285" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B286" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C286" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D286" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E286" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B287" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C287" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D287" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E287" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B288" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C288" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D288" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E288" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B289" t="s">
-        <v>287</v>
+        <v>326</v>
       </c>
       <c r="C289" t="s">
-        <v>288</v>
+        <v>327</v>
       </c>
       <c r="D289" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E289" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B290" t="s">
-        <v>326</v>
+        <v>290</v>
       </c>
       <c r="C290" t="s">
-        <v>327</v>
+        <v>291</v>
       </c>
       <c r="D290" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E290" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B291" t="s">
-        <v>326</v>
+        <v>290</v>
       </c>
       <c r="C291" t="s">
-        <v>327</v>
+        <v>291</v>
       </c>
       <c r="D291" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E291" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B292" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C292" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D292" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E292" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B293" t="s">
-        <v>287</v>
+        <v>332</v>
       </c>
       <c r="C293" t="s">
-        <v>288</v>
+        <v>333</v>
       </c>
       <c r="D293" t="s">
-        <v>289</v>
+        <v>334</v>
       </c>
       <c r="E293" t="s">
-        <v>290</v>
+        <v>335</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="B294" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="C294" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D294" t="s">
         <v>334</v>
@@ -6771,13 +6774,13 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B295" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="C295" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="D295" t="s">
         <v>334</v>
@@ -6788,7 +6791,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B296" t="s">
         <v>340</v>
@@ -6805,7 +6808,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B297" t="s">
         <v>340</v>
@@ -6822,7 +6825,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B298" t="s">
         <v>340</v>
@@ -6839,7 +6842,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B299" t="s">
         <v>340</v>
@@ -6856,7 +6859,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B300" t="s">
         <v>340</v>
@@ -6873,7 +6876,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B301" t="s">
         <v>340</v>
@@ -6890,7 +6893,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B302" t="s">
         <v>340</v>
@@ -6907,7 +6910,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B303" t="s">
         <v>340</v>
@@ -6924,7 +6927,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B304" t="s">
         <v>340</v>
@@ -6941,7 +6944,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B305" t="s">
         <v>340</v>
@@ -6958,7 +6961,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B306" t="s">
         <v>340</v>
@@ -6975,7 +6978,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B307" t="s">
         <v>340</v>
@@ -6992,7 +6995,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B308" t="s">
         <v>340</v>
@@ -7009,7 +7012,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B309" t="s">
         <v>340</v>
@@ -7026,7 +7029,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B310" t="s">
         <v>340</v>
@@ -7043,7 +7046,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B311" t="s">
         <v>340</v>
@@ -7060,7 +7063,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B312" t="s">
         <v>340</v>
@@ -7077,13 +7080,13 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B313" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="C313" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="D313" t="s">
         <v>334</v>
@@ -7094,7 +7097,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B314" t="s">
         <v>332</v>
@@ -7111,7 +7114,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B315" t="s">
         <v>332</v>
@@ -7128,7 +7131,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B316" t="s">
         <v>332</v>
@@ -7145,7 +7148,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B317" t="s">
         <v>332</v>
@@ -7162,7 +7165,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B318" t="s">
         <v>332</v>
@@ -7179,7 +7182,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B319" t="s">
         <v>332</v>
@@ -7196,7 +7199,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B320" t="s">
         <v>332</v>
@@ -7213,13 +7216,13 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B321" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="C321" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D321" t="s">
         <v>334</v>
@@ -7233,10 +7236,10 @@
         <v>367</v>
       </c>
       <c r="B322" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="C322" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D322" t="s">
         <v>334</v>
@@ -7247,13 +7250,13 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B323" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="C323" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D323" t="s">
         <v>334</v>
@@ -7264,7 +7267,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B324" t="s">
         <v>337</v>
@@ -7281,7 +7284,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B325" t="s">
         <v>337</v>
@@ -7298,7 +7301,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B326" t="s">
         <v>337</v>
@@ -7315,13 +7318,13 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B327" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="C327" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D327" t="s">
         <v>334</v>
@@ -7332,7 +7335,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B328" t="s">
         <v>332</v>
@@ -7349,7 +7352,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B329" t="s">
         <v>332</v>
@@ -7366,7 +7369,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B330" t="s">
         <v>332</v>
@@ -7383,7 +7386,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B331" t="s">
         <v>332</v>
@@ -7400,7 +7403,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B332" t="s">
         <v>332</v>
@@ -7417,7 +7420,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B333" t="s">
         <v>332</v>
@@ -7434,7 +7437,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B334" t="s">
         <v>332</v>
@@ -7451,7 +7454,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B335" t="s">
         <v>332</v>
@@ -7468,7 +7471,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B336" t="s">
         <v>332</v>
@@ -7485,7 +7488,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B337" t="s">
         <v>332</v>
@@ -7502,13 +7505,13 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B338" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="C338" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="D338" t="s">
         <v>334</v>
@@ -7519,7 +7522,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B339" t="s">
         <v>337</v>
@@ -7536,7 +7539,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B340" t="s">
         <v>337</v>
@@ -7553,7 +7556,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B341" t="s">
         <v>337</v>
@@ -7570,7 +7573,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B342" t="s">
         <v>337</v>
@@ -7587,7 +7590,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B343" t="s">
         <v>337</v>
@@ -7604,7 +7607,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B344" t="s">
         <v>337</v>
@@ -7621,7 +7624,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B345" t="s">
         <v>337</v>
@@ -7638,7 +7641,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B346" t="s">
         <v>337</v>
@@ -7655,7 +7658,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B347" t="s">
         <v>337</v>
@@ -7672,7 +7675,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B348" t="s">
         <v>337</v>
@@ -7689,7 +7692,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B349" t="s">
         <v>337</v>
@@ -7706,7 +7709,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B350" t="s">
         <v>337</v>
@@ -7723,7 +7726,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B351" t="s">
         <v>337</v>
@@ -7740,7 +7743,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B352" t="s">
         <v>337</v>
@@ -7757,7 +7760,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B353" t="s">
         <v>337</v>
@@ -7774,7 +7777,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B354" t="s">
         <v>337</v>
@@ -7791,7 +7794,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B355" t="s">
         <v>337</v>
@@ -7808,7 +7811,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B356" t="s">
         <v>337</v>
@@ -7825,7 +7828,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B357" t="s">
         <v>337</v>
@@ -7842,7 +7845,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B358" t="s">
         <v>337</v>
@@ -7859,7 +7862,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B359" t="s">
         <v>337</v>
@@ -7876,7 +7879,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B360" t="s">
         <v>337</v>
@@ -7893,7 +7896,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B361" t="s">
         <v>337</v>
@@ -7910,13 +7913,13 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B362" t="s">
-        <v>337</v>
+        <v>408</v>
       </c>
       <c r="C362" t="s">
-        <v>338</v>
+        <v>409</v>
       </c>
       <c r="D362" t="s">
         <v>334</v>
@@ -7927,7 +7930,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="B363" t="s">
         <v>408</v>
@@ -7944,7 +7947,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B364" t="s">
         <v>408</v>
@@ -7961,7 +7964,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B365" t="s">
         <v>408</v>
@@ -7978,7 +7981,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B366" t="s">
         <v>408</v>
@@ -7995,7 +7998,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="B367" t="s">
         <v>408</v>
@@ -8012,7 +8015,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B368" t="s">
         <v>408</v>
@@ -8029,7 +8032,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="B369" t="s">
         <v>408</v>
@@ -8046,7 +8049,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B370" t="s">
         <v>408</v>
@@ -8063,7 +8066,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B371" t="s">
         <v>408</v>
@@ -8080,7 +8083,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B372" t="s">
         <v>408</v>
@@ -8097,7 +8100,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B373" t="s">
         <v>408</v>
@@ -8114,7 +8117,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B374" t="s">
         <v>408</v>
@@ -8131,7 +8134,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="B375" t="s">
         <v>408</v>
@@ -8148,7 +8151,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B376" t="s">
         <v>408</v>
@@ -8165,7 +8168,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B377" t="s">
         <v>408</v>
@@ -8182,7 +8185,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="B378" t="s">
         <v>408</v>
@@ -8199,7 +8202,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="B379" t="s">
         <v>408</v>
@@ -8216,7 +8219,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B380" t="s">
         <v>408</v>
@@ -8233,41 +8236,41 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B381" t="s">
-        <v>408</v>
+        <v>326</v>
       </c>
       <c r="C381" t="s">
-        <v>409</v>
+        <v>327</v>
       </c>
       <c r="D381" t="s">
-        <v>334</v>
+        <v>292</v>
       </c>
       <c r="E381" t="s">
-        <v>335</v>
+        <v>293</v>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B382" t="s">
-        <v>326</v>
+        <v>430</v>
       </c>
       <c r="C382" t="s">
-        <v>327</v>
+        <v>431</v>
       </c>
       <c r="D382" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E382" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B383" t="s">
         <v>430</v>
@@ -8276,32 +8279,32 @@
         <v>431</v>
       </c>
       <c r="D383" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E383" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B384" t="s">
-        <v>430</v>
+        <v>326</v>
       </c>
       <c r="C384" t="s">
-        <v>431</v>
+        <v>327</v>
       </c>
       <c r="D384" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E384" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="B385" t="s">
         <v>326</v>
@@ -8310,15 +8313,15 @@
         <v>327</v>
       </c>
       <c r="D385" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E385" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B386" t="s">
         <v>326</v>
@@ -8327,15 +8330,15 @@
         <v>327</v>
       </c>
       <c r="D386" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E386" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B387" t="s">
         <v>326</v>
@@ -8344,15 +8347,15 @@
         <v>327</v>
       </c>
       <c r="D387" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E387" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="B388" t="s">
         <v>326</v>
@@ -8361,15 +8364,15 @@
         <v>327</v>
       </c>
       <c r="D388" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E388" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B389" t="s">
         <v>326</v>
@@ -8378,15 +8381,15 @@
         <v>327</v>
       </c>
       <c r="D389" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E389" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="B390" t="s">
         <v>326</v>
@@ -8395,15 +8398,15 @@
         <v>327</v>
       </c>
       <c r="D390" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E390" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="B391" t="s">
         <v>326</v>
@@ -8412,32 +8415,32 @@
         <v>327</v>
       </c>
       <c r="D391" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E391" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B392" t="s">
-        <v>326</v>
+        <v>430</v>
       </c>
       <c r="C392" t="s">
-        <v>327</v>
+        <v>431</v>
       </c>
       <c r="D392" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E392" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B393" t="s">
         <v>326</v>
@@ -8446,32 +8449,32 @@
         <v>327</v>
       </c>
       <c r="D393" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E393" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B394" t="s">
-        <v>430</v>
+        <v>326</v>
       </c>
       <c r="C394" t="s">
-        <v>431</v>
+        <v>327</v>
       </c>
       <c r="D394" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E394" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="B395" t="s">
         <v>326</v>
@@ -8480,15 +8483,15 @@
         <v>327</v>
       </c>
       <c r="D395" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E395" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="B396" t="s">
         <v>326</v>
@@ -8497,15 +8500,15 @@
         <v>327</v>
       </c>
       <c r="D396" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E396" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B397" t="s">
         <v>326</v>
@@ -8514,15 +8517,15 @@
         <v>327</v>
       </c>
       <c r="D397" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E397" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B398" t="s">
         <v>326</v>
@@ -8531,15 +8534,15 @@
         <v>327</v>
       </c>
       <c r="D398" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E398" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B399" t="s">
         <v>326</v>
@@ -8548,15 +8551,15 @@
         <v>327</v>
       </c>
       <c r="D399" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E399" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B400" t="s">
         <v>326</v>
@@ -8565,15 +8568,15 @@
         <v>327</v>
       </c>
       <c r="D400" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E400" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B401" t="s">
         <v>326</v>
@@ -8582,15 +8585,15 @@
         <v>327</v>
       </c>
       <c r="D401" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E401" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B402" t="s">
         <v>326</v>
@@ -8599,15 +8602,15 @@
         <v>327</v>
       </c>
       <c r="D402" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E402" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B403" t="s">
         <v>326</v>
@@ -8616,15 +8619,15 @@
         <v>327</v>
       </c>
       <c r="D403" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E403" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B404" t="s">
         <v>326</v>
@@ -8633,15 +8636,15 @@
         <v>327</v>
       </c>
       <c r="D404" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E404" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B405" t="s">
         <v>326</v>
@@ -8650,49 +8653,49 @@
         <v>327</v>
       </c>
       <c r="D405" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E405" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="B406" t="s">
-        <v>326</v>
+        <v>430</v>
       </c>
       <c r="C406" t="s">
-        <v>327</v>
+        <v>431</v>
       </c>
       <c r="D406" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E406" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B407" t="s">
-        <v>326</v>
+        <v>430</v>
       </c>
       <c r="C407" t="s">
-        <v>327</v>
+        <v>431</v>
       </c>
       <c r="D407" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E407" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="B408" t="s">
         <v>430</v>
@@ -8701,15 +8704,15 @@
         <v>431</v>
       </c>
       <c r="D408" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E408" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B409" t="s">
         <v>430</v>
@@ -8718,15 +8721,15 @@
         <v>431</v>
       </c>
       <c r="D409" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E409" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="B410" t="s">
         <v>430</v>
@@ -8735,15 +8738,15 @@
         <v>431</v>
       </c>
       <c r="D410" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E410" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B411" t="s">
         <v>430</v>
@@ -8752,15 +8755,15 @@
         <v>431</v>
       </c>
       <c r="D411" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E411" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="B412" t="s">
         <v>430</v>
@@ -8769,15 +8772,15 @@
         <v>431</v>
       </c>
       <c r="D412" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E412" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="B413" t="s">
         <v>430</v>
@@ -8786,32 +8789,32 @@
         <v>431</v>
       </c>
       <c r="D413" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E413" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B414" t="s">
-        <v>326</v>
+        <v>430</v>
       </c>
       <c r="C414" t="s">
-        <v>327</v>
+        <v>431</v>
       </c>
       <c r="D414" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E414" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B415" t="s">
         <v>430</v>
@@ -8820,15 +8823,15 @@
         <v>431</v>
       </c>
       <c r="D415" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E415" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B416" t="s">
         <v>430</v>
@@ -8837,15 +8840,15 @@
         <v>431</v>
       </c>
       <c r="D416" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E416" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B417" t="s">
         <v>430</v>
@@ -8854,15 +8857,15 @@
         <v>431</v>
       </c>
       <c r="D417" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E417" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B418" t="s">
         <v>430</v>
@@ -8871,15 +8874,15 @@
         <v>431</v>
       </c>
       <c r="D418" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E418" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B419" t="s">
         <v>430</v>
@@ -8888,15 +8891,15 @@
         <v>431</v>
       </c>
       <c r="D419" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E419" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B420" t="s">
         <v>430</v>
@@ -8905,15 +8908,15 @@
         <v>431</v>
       </c>
       <c r="D420" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E420" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B421" t="s">
         <v>430</v>
@@ -8922,15 +8925,15 @@
         <v>431</v>
       </c>
       <c r="D421" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E421" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B422" t="s">
         <v>430</v>
@@ -8939,15 +8942,15 @@
         <v>431</v>
       </c>
       <c r="D422" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E422" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B423" t="s">
         <v>430</v>
@@ -8956,15 +8959,15 @@
         <v>431</v>
       </c>
       <c r="D423" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E423" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B424" t="s">
         <v>430</v>
@@ -8973,15 +8976,15 @@
         <v>431</v>
       </c>
       <c r="D424" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E424" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B425" t="s">
         <v>430</v>
@@ -8990,32 +8993,32 @@
         <v>431</v>
       </c>
       <c r="D425" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E425" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B426" t="s">
-        <v>430</v>
+        <v>326</v>
       </c>
       <c r="C426" t="s">
-        <v>431</v>
+        <v>327</v>
       </c>
       <c r="D426" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E426" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B427" t="s">
         <v>430</v>
@@ -9024,44 +9027,44 @@
         <v>431</v>
       </c>
       <c r="D427" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E427" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="B428" t="s">
-        <v>430</v>
+        <v>326</v>
       </c>
       <c r="C428" t="s">
-        <v>431</v>
+        <v>327</v>
       </c>
       <c r="D428" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E428" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B429" t="s">
-        <v>326</v>
+        <v>290</v>
       </c>
       <c r="C429" t="s">
-        <v>327</v>
+        <v>291</v>
       </c>
       <c r="D429" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E429" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
   </sheetData>

</xml_diff>